<commit_message>
adding general information and bankflow comparison
</commit_message>
<xml_diff>
--- a/fluxo_de_caixa.xlsx
+++ b/fluxo_de_caixa.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="296">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="281">
   <si>
     <t>Conta</t>
   </si>
@@ -49,12 +49,6 @@
     <t>Mensalidade Inf 3 e 4</t>
   </si>
   <si>
-    <t>1.12.005</t>
-  </si>
-  <si>
-    <t>Mens. Integral 10h- Infan. 3 e 4</t>
-  </si>
-  <si>
     <t>1.13.001</t>
   </si>
   <si>
@@ -67,12 +61,6 @@
     <t>Matrícula Fund 1</t>
   </si>
   <si>
-    <t>1.13.003</t>
-  </si>
-  <si>
-    <t>Mens. Integral 6h - Fund I</t>
-  </si>
-  <si>
     <t>1.13.005</t>
   </si>
   <si>
@@ -133,10 +121,10 @@
     <t>Ballet</t>
   </si>
   <si>
-    <t>1.21.005</t>
-  </si>
-  <si>
-    <t>Futsal</t>
+    <t>1.21.008</t>
+  </si>
+  <si>
+    <t>Armário</t>
   </si>
   <si>
     <t>1.21.009</t>
@@ -145,12 +133,6 @@
     <t>Natação</t>
   </si>
   <si>
-    <t>1.21.014</t>
-  </si>
-  <si>
-    <t>Karatê</t>
-  </si>
-  <si>
     <t>122.000</t>
   </si>
   <si>
@@ -163,12 +145,6 @@
     <t>Apostilas Anglo e complementares</t>
   </si>
   <si>
-    <t>1.22.003</t>
-  </si>
-  <si>
-    <t>Avaliação substitutiva</t>
-  </si>
-  <si>
     <t>1.22.006</t>
   </si>
   <si>
@@ -181,12 +157,6 @@
     <t>CURSOS LIVRES</t>
   </si>
   <si>
-    <t>1.23.005</t>
-  </si>
-  <si>
-    <t>Curso de Férias</t>
-  </si>
-  <si>
     <t>124.000</t>
   </si>
   <si>
@@ -199,24 +169,12 @@
     <t>Revenda de lanches</t>
   </si>
   <si>
-    <t>1.24.007</t>
-  </si>
-  <si>
-    <t>Revenda Almoço</t>
-  </si>
-  <si>
     <t>125.000</t>
   </si>
   <si>
     <t>EVENTOS</t>
   </si>
   <si>
-    <t>1.25.003</t>
-  </si>
-  <si>
-    <t>Passeios</t>
-  </si>
-  <si>
     <t>1.25.010</t>
   </si>
   <si>
@@ -229,12 +187,6 @@
     <t>Convites extras formatura</t>
   </si>
   <si>
-    <t>1.25.012</t>
-  </si>
-  <si>
-    <t>Foto/filmag. formatura</t>
-  </si>
-  <si>
     <t>1.25.015</t>
   </si>
   <si>
@@ -313,12 +265,6 @@
     <t>Acordo mensalidade</t>
   </si>
   <si>
-    <t>1.30.002</t>
-  </si>
-  <si>
-    <t>Devolução ou reembolso</t>
-  </si>
-  <si>
     <t>200.000</t>
   </si>
   <si>
@@ -331,73 +277,73 @@
     <t>SERVIÇOS BÁSICOS</t>
   </si>
   <si>
-    <t xml:space="preserve">2.01.001 </t>
+    <t>2.01.001</t>
   </si>
   <si>
     <t>Água unidade 1</t>
   </si>
   <si>
-    <t xml:space="preserve">2.01.002 </t>
+    <t>2.01.002</t>
   </si>
   <si>
     <t>Água unidade 2</t>
   </si>
   <si>
-    <t xml:space="preserve">2.01.003 </t>
+    <t>2.01.003</t>
   </si>
   <si>
     <t>Água unidade 3</t>
   </si>
   <si>
-    <t xml:space="preserve">2.01.004 </t>
+    <t>2.01.004</t>
   </si>
   <si>
     <t>Luz unidade 1</t>
   </si>
   <si>
-    <t xml:space="preserve">2.01.005 </t>
+    <t>2.01.005</t>
   </si>
   <si>
     <t>Luz unidade 2</t>
   </si>
   <si>
-    <t xml:space="preserve">2.01.006 </t>
+    <t>2.01.006</t>
   </si>
   <si>
     <t>Luz unidade 3</t>
   </si>
   <si>
-    <t xml:space="preserve">2.01.008 </t>
+    <t>2.01.008</t>
   </si>
   <si>
     <t>Net unidade 1</t>
   </si>
   <si>
-    <t xml:space="preserve">2.01.011 </t>
+    <t>2.01.011</t>
   </si>
   <si>
     <t>Celulares comerciais</t>
   </si>
   <si>
-    <t xml:space="preserve">2.01.012 </t>
+    <t>2.01.012</t>
   </si>
   <si>
     <t>Despesa de Aluguel</t>
   </si>
   <si>
-    <t xml:space="preserve">2.01.013 </t>
+    <t>2.01.013</t>
   </si>
   <si>
     <t>Vivo Unidade 2</t>
   </si>
   <si>
-    <t xml:space="preserve">2.01.014 </t>
+    <t>2.01.014</t>
   </si>
   <si>
     <t>Vivo Unidade 1</t>
   </si>
   <si>
-    <t xml:space="preserve">2.01.015 </t>
+    <t>2.01.015</t>
   </si>
   <si>
     <t>Vivo Unidade 3</t>
@@ -409,61 +355,67 @@
     <t>DESPESAS GERAIS</t>
   </si>
   <si>
-    <t xml:space="preserve">2.02.101 </t>
-  </si>
-  <si>
-    <t>Jornal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.02.102 </t>
+    <t>2.02.102</t>
   </si>
   <si>
     <t>Materiais esportivos</t>
   </si>
   <si>
-    <t xml:space="preserve">2.02.200 </t>
+    <t>2.02.105</t>
+  </si>
+  <si>
+    <t>Material laboratório</t>
+  </si>
+  <si>
+    <t>2.02.200</t>
   </si>
   <si>
     <t>DESP. MANUTENÇÃO E CONSERVAÇÃO</t>
   </si>
   <si>
-    <t xml:space="preserve">2.02.204 </t>
+    <t>2.02.201</t>
+  </si>
+  <si>
+    <t>Outros Materiais de Manutenção</t>
+  </si>
+  <si>
+    <t>2.02.202</t>
+  </si>
+  <si>
+    <t>Materiais elétricos</t>
+  </si>
+  <si>
+    <t>2.02.203</t>
+  </si>
+  <si>
+    <t>Materiais de construção</t>
+  </si>
+  <si>
+    <t>2.02.204</t>
   </si>
   <si>
     <t>Manutenção de equipamentos</t>
   </si>
   <si>
-    <t xml:space="preserve">2.02.301 </t>
+    <t>2.02.301</t>
   </si>
   <si>
     <t>Material de cozinha</t>
   </si>
   <si>
-    <t xml:space="preserve">2.02.302 </t>
+    <t>2.02.302</t>
   </si>
   <si>
     <t>Material de limpeza e higiene</t>
   </si>
   <si>
-    <t xml:space="preserve">2.02.602 </t>
-  </si>
-  <si>
-    <t>Gasolina e estacionamento</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.02.603 </t>
+    <t>2.02.603</t>
   </si>
   <si>
     <t>Lanches e refeições</t>
   </si>
   <si>
-    <t xml:space="preserve">2.02.604 </t>
-  </si>
-  <si>
-    <t>Farmácia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.02.610 </t>
+    <t>2.02.610</t>
   </si>
   <si>
     <t>Sieeesp</t>
@@ -475,10 +427,7 @@
     <t>Apostilas Anglo e Complementares</t>
   </si>
   <si>
-    <t xml:space="preserve">2.02.103 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.02.104 </t>
+    <t>2.02.104</t>
   </si>
   <si>
     <t>Material pedagógico</t>
@@ -490,127 +439,121 @@
     <t>SERVIÇOS CONTRATADOS</t>
   </si>
   <si>
-    <t xml:space="preserve">2.03.001 </t>
+    <t>2.03.001</t>
   </si>
   <si>
     <t>Serviço de monitor./alarme 1 e 2</t>
   </si>
   <si>
-    <t xml:space="preserve">2.03.002 </t>
-  </si>
-  <si>
-    <t>Serviço de monitor./alarme 3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.03.004 </t>
+    <t>2.03.004</t>
   </si>
   <si>
     <t>Serviço de aulas de música</t>
   </si>
   <si>
-    <t xml:space="preserve">2.03.007 </t>
+    <t>2.03.007</t>
   </si>
   <si>
     <t>Serviço Arteterapia</t>
   </si>
   <si>
-    <t xml:space="preserve">2.03.010 </t>
+    <t>2.03.009</t>
+  </si>
+  <si>
+    <t>Serviços de informática</t>
+  </si>
+  <si>
+    <t>2.03.010</t>
   </si>
   <si>
     <t>Serviços de Contabilidade 1 e 2</t>
   </si>
   <si>
-    <t xml:space="preserve">2.03.011 </t>
+    <t>2.03.011</t>
   </si>
   <si>
     <t>Serviços de Contabilidade 3</t>
   </si>
   <si>
-    <t xml:space="preserve">2.03.012 </t>
+    <t>2.03.012</t>
   </si>
   <si>
     <t>Serviços de consulta PF e PJ</t>
   </si>
   <si>
-    <t xml:space="preserve">2.03.014 </t>
+    <t>2.03.014</t>
   </si>
   <si>
     <t>Serviços advocatícios</t>
   </si>
   <si>
-    <t xml:space="preserve">2.03.015 </t>
+    <t>2.03.015</t>
   </si>
   <si>
     <t>Serviço de marcenaria</t>
   </si>
   <si>
-    <t xml:space="preserve">2.03.016 </t>
+    <t>2.03.016</t>
   </si>
   <si>
     <t>Serviço propaganda e publicidade</t>
   </si>
   <si>
-    <t xml:space="preserve">2.03.021 </t>
+    <t>2.03.021</t>
   </si>
   <si>
     <t>Serviços de medicina do trabalho</t>
   </si>
   <si>
-    <t xml:space="preserve">2.03.022 </t>
+    <t>2.03.022</t>
   </si>
   <si>
     <t>Serviço agenda eletrônica</t>
   </si>
   <si>
-    <t xml:space="preserve">2.03.023 </t>
-  </si>
-  <si>
-    <t>Serviço de aulas de inglês e esp</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.03.024 </t>
+    <t>2.03.024</t>
   </si>
   <si>
     <t>Serviços gráficos (copiadoras)</t>
   </si>
   <si>
-    <t xml:space="preserve">2.03.026 </t>
+    <t>2.03.026</t>
   </si>
   <si>
     <t>Serviços de robótica</t>
   </si>
   <si>
-    <t xml:space="preserve">2.03.027 </t>
+    <t>2.03.027</t>
   </si>
   <si>
     <t>Serviços de psicologia</t>
   </si>
   <si>
-    <t xml:space="preserve">2.03.028 </t>
+    <t>2.03.028</t>
   </si>
   <si>
     <t>Serviços balé e dança educativa</t>
   </si>
   <si>
-    <t xml:space="preserve">2.03.029 </t>
+    <t>2.03.029</t>
   </si>
   <si>
     <t>Serviços de assessoria</t>
   </si>
   <si>
-    <t xml:space="preserve">2.03.031 </t>
+    <t>2.03.031</t>
   </si>
   <si>
     <t>Serviços de natação</t>
   </si>
   <si>
-    <t xml:space="preserve">2.03.032 </t>
+    <t>2.03.032</t>
   </si>
   <si>
     <t>Serviços de contrato digital</t>
   </si>
   <si>
-    <t xml:space="preserve">2.03.033 </t>
+    <t>2.03.033</t>
   </si>
   <si>
     <t>Serviços de Karatê</t>
@@ -622,85 +565,103 @@
     <t>SALÁRIOS E ENCARGOS</t>
   </si>
   <si>
-    <t xml:space="preserve">2.04.001 </t>
+    <t>2.04.001</t>
   </si>
   <si>
     <t>Salários professores</t>
   </si>
   <si>
-    <t xml:space="preserve">2.04.002 </t>
+    <t>2.04.002</t>
   </si>
   <si>
     <t>Salários administrativos</t>
   </si>
   <si>
-    <t xml:space="preserve">2.04.007 </t>
+    <t>2.04.007</t>
   </si>
   <si>
     <t>Fgts unidade 1</t>
   </si>
   <si>
-    <t xml:space="preserve">2.04.008 </t>
+    <t>2.04.008</t>
   </si>
   <si>
     <t>Fgts unidade 2</t>
   </si>
   <si>
-    <t xml:space="preserve">2.04.009 </t>
+    <t>2.04.009</t>
   </si>
   <si>
     <t>Fgts unidade 3</t>
   </si>
   <si>
-    <t xml:space="preserve">2.04.010 </t>
+    <t>2.04.010</t>
   </si>
   <si>
     <t>Darf 561</t>
   </si>
   <si>
-    <t xml:space="preserve">2.04.020 </t>
+    <t>2.04.019</t>
+  </si>
+  <si>
+    <t>Rescisão funcionário</t>
+  </si>
+  <si>
+    <t>2.04.020</t>
   </si>
   <si>
     <t>Sinpro</t>
   </si>
   <si>
-    <t xml:space="preserve">2.04.021 </t>
+    <t>2.04.021</t>
   </si>
   <si>
     <t>Saaesp</t>
   </si>
   <si>
-    <t xml:space="preserve">2.04.023 </t>
+    <t>2.04.023</t>
   </si>
   <si>
     <t>Seguro funcionários</t>
   </si>
   <si>
-    <t xml:space="preserve">2.04.024 </t>
+    <t>2.04.024</t>
   </si>
   <si>
     <t>Vale transporte</t>
   </si>
   <si>
-    <t xml:space="preserve">2.04.025 </t>
+    <t>2.04.025</t>
   </si>
   <si>
     <t>Vale alimentação</t>
   </si>
   <si>
+    <t>2.04.026</t>
+  </si>
+  <si>
+    <t>Darf 0588</t>
+  </si>
+  <si>
     <t>205.000</t>
   </si>
   <si>
     <t>BENEFÍCIOS</t>
   </si>
   <si>
-    <t xml:space="preserve">2.05.004 </t>
-  </si>
-  <si>
-    <t>Comissão de matrícula</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.05.008 </t>
+    <t>2.05.005</t>
+  </si>
+  <si>
+    <t>Cursos para professor</t>
+  </si>
+  <si>
+    <t>2.05.007</t>
+  </si>
+  <si>
+    <t>Meritocracia</t>
+  </si>
+  <si>
+    <t>2.05.008</t>
   </si>
   <si>
     <t>Uniforme funcionário</t>
@@ -712,16 +673,34 @@
     <t>ESTAGIARIOS</t>
   </si>
   <si>
-    <t xml:space="preserve">2.06.003 </t>
+    <t>2.06.003</t>
   </si>
   <si>
     <t>Bolsa auxilio estagiários</t>
   </si>
   <si>
+    <t>2.06.005</t>
+  </si>
+  <si>
+    <t>Seguro estagiários</t>
+  </si>
+  <si>
     <t>207.000</t>
   </si>
   <si>
-    <t xml:space="preserve">2.07.003 </t>
+    <t>2.07.001</t>
+  </si>
+  <si>
+    <t>Multas a pagar</t>
+  </si>
+  <si>
+    <t>2.07.002</t>
+  </si>
+  <si>
+    <t>Juros a pagar</t>
+  </si>
+  <si>
+    <t>2.07.003</t>
   </si>
   <si>
     <t>Tarifas bancárias</t>
@@ -733,31 +712,19 @@
     <t>TRIBUTÁRIAS</t>
   </si>
   <si>
-    <t xml:space="preserve">2.12.101 </t>
-  </si>
-  <si>
-    <t>Iptu unidade 3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.12.102 </t>
-  </si>
-  <si>
-    <t>Iptu unidade 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.12.103 </t>
-  </si>
-  <si>
-    <t>Iptu unidade 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.12.201 </t>
+    <t>2.12.201</t>
   </si>
   <si>
     <t>Simples Nacional</t>
   </si>
   <si>
-    <t xml:space="preserve">2.12.304 </t>
+    <t>2.12.202</t>
+  </si>
+  <si>
+    <t>IOF</t>
+  </si>
+  <si>
+    <t>2.12.304</t>
   </si>
   <si>
     <t>ISS s/ PJ</t>
@@ -769,7 +736,19 @@
     <t>SEGUROS</t>
   </si>
   <si>
-    <t xml:space="preserve">2.14.004 </t>
+    <t>2.14.001</t>
+  </si>
+  <si>
+    <t>Despesa c/ Seguro predial uni. 3</t>
+  </si>
+  <si>
+    <t>2.14.002</t>
+  </si>
+  <si>
+    <t>Despesa c/ Seguro predial uni. 1</t>
+  </si>
+  <si>
+    <t>2.14.004</t>
   </si>
   <si>
     <t>Despesa c/ Seguro educacional</t>
@@ -781,13 +760,19 @@
     <t>REMATRICULA</t>
   </si>
   <si>
+    <t>2.16.002</t>
+  </si>
+  <si>
+    <t>Rematrícula custo com brindes</t>
+  </si>
+  <si>
     <t>217.000</t>
   </si>
   <si>
     <t>SÓCIAS</t>
   </si>
   <si>
-    <t xml:space="preserve">2.17.001 </t>
+    <t>2.17.001</t>
   </si>
   <si>
     <t>Despesas sócias</t>
@@ -799,76 +784,34 @@
     <t>CUSTO REVENDAS DIVERSAS</t>
   </si>
   <si>
-    <t xml:space="preserve">2.20.001 </t>
+    <t>2.20.001</t>
   </si>
   <si>
     <t>Lanches para revenda</t>
   </si>
   <si>
+    <t>2.20.002</t>
+  </si>
+  <si>
+    <t>Sucos para revenda</t>
+  </si>
+  <si>
     <t>230.000</t>
   </si>
   <si>
-    <t xml:space="preserve">2.30.101 </t>
-  </si>
-  <si>
-    <t>Formatura - Infantil 4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.30.102 </t>
+    <t>2.30.102</t>
   </si>
   <si>
     <t>Formatura 9ª ano</t>
   </si>
   <si>
-    <t xml:space="preserve">2.30.200 </t>
+    <t>2.30.200</t>
   </si>
   <si>
     <t>MOSTRA DE DANÇA</t>
   </si>
   <si>
-    <t xml:space="preserve">2.30.203 </t>
-  </si>
-  <si>
-    <t>Desp. div. Mostra de Dança</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.30.204 </t>
-  </si>
-  <si>
-    <t>Teatro Mostra de Dança</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.30.401 </t>
-  </si>
-  <si>
-    <t>Custo diversos Olimpiada</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.30.501 </t>
-  </si>
-  <si>
-    <t>Custo acampamento</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.30.601 </t>
-  </si>
-  <si>
-    <t>Passeios diversos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.30.801 </t>
-  </si>
-  <si>
-    <t>Mostra Cultural Uni 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.31.101 </t>
-  </si>
-  <si>
-    <t>Confraternização funcionários</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.31.102 </t>
+    <t>2.31.102</t>
   </si>
   <si>
     <t>Brindes e presentes</t>
@@ -880,28 +823,40 @@
     <t>IMOBILIZADO</t>
   </si>
   <si>
-    <t xml:space="preserve">2.40.001 </t>
+    <t>2.40.001</t>
   </si>
   <si>
     <t>Sophia - Sistema de Gestão</t>
   </si>
   <si>
-    <t xml:space="preserve">2.40.002 </t>
+    <t>2.40.002</t>
   </si>
   <si>
     <t>Móveis e utensílios</t>
   </si>
   <si>
-    <t xml:space="preserve">2.40.005 </t>
+    <t>2.40.005</t>
   </si>
   <si>
     <t>Empréstimo a pagar</t>
   </si>
   <si>
-    <t xml:space="preserve">2.40.006 </t>
+    <t>2.40.006</t>
   </si>
   <si>
     <t>Máquinas e equipamentos</t>
+  </si>
+  <si>
+    <t>Descrição</t>
+  </si>
+  <si>
+    <t>Sophia</t>
+  </si>
+  <si>
+    <t>Extrato</t>
+  </si>
+  <si>
+    <t>Diferença</t>
   </si>
 </sst>
 </file>
@@ -911,7 +866,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.00"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -927,8 +882,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -944,6 +907,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFD9E1F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF4B942"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -975,13 +950,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="1" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="2" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1276,12 +1254,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C149"/>
+  <dimension ref="A1:E143"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="18.7109375" customWidth="1"/>
     <col min="2" max="2" width="45.7109375" customWidth="1"/>
-    <col min="3" max="3" width="16.7109375" customWidth="1"/>
+    <col min="3" max="5" width="16.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1303,7 +1281,7 @@
         <v>4</v>
       </c>
       <c r="C2" s="3">
-        <v>441711.3800000001</v>
+        <v>379129.2</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -1314,7 +1292,7 @@
         <v>6</v>
       </c>
       <c r="C3" s="3">
-        <v>346020.2068</v>
+        <v>286536.85</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -1325,7 +1303,7 @@
         <v>8</v>
       </c>
       <c r="C4" s="5">
-        <v>457.52</v>
+        <v>297.52</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -1336,7 +1314,7 @@
         <v>10</v>
       </c>
       <c r="C5" s="5">
-        <v>432.52</v>
+        <v>254.43</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -1347,7 +1325,7 @@
         <v>12</v>
       </c>
       <c r="C6" s="5">
-        <v>120</v>
+        <v>2644.3552</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -1358,7 +1336,7 @@
         <v>14</v>
       </c>
       <c r="C7" s="5">
-        <v>4885.2888</v>
+        <v>707.3848</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -1369,7 +1347,7 @@
         <v>16</v>
       </c>
       <c r="C8" s="5">
-        <v>465.308</v>
+        <v>1926.54</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -1380,7 +1358,7 @@
         <v>18</v>
       </c>
       <c r="C9" s="5">
-        <v>67.8</v>
+        <v>851.88</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -1391,7 +1369,7 @@
         <v>20</v>
       </c>
       <c r="C10" s="5">
-        <v>422.04</v>
+        <v>169.52</v>
       </c>
     </row>
     <row r="11" spans="1:3">
@@ -1402,7 +1380,7 @@
         <v>22</v>
       </c>
       <c r="C11" s="5">
-        <v>32552.13</v>
+        <v>10958.36</v>
       </c>
     </row>
     <row r="12" spans="1:3">
@@ -1413,7 +1391,7 @@
         <v>24</v>
       </c>
       <c r="C12" s="5">
-        <v>1804.26</v>
+        <v>49902.27</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -1424,7 +1402,7 @@
         <v>26</v>
       </c>
       <c r="C13" s="5">
-        <v>6894.23</v>
+        <v>47333.81</v>
       </c>
     </row>
     <row r="14" spans="1:3">
@@ -1435,51 +1413,51 @@
         <v>28</v>
       </c>
       <c r="C14" s="5">
-        <v>66093.87</v>
+        <v>171490.78</v>
       </c>
     </row>
     <row r="15" spans="1:3">
-      <c r="A15" s="4" t="s">
+      <c r="A15" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C15" s="5">
-        <v>15605.47</v>
+      <c r="C15" s="3">
+        <v>91774.29000000001</v>
       </c>
     </row>
     <row r="16" spans="1:3">
-      <c r="A16" s="4" t="s">
+      <c r="A16" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="B16" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C16" s="5">
-        <v>216219.77</v>
+      <c r="C16" s="3">
+        <v>5015.66</v>
       </c>
     </row>
     <row r="17" spans="1:3">
-      <c r="A17" s="2" t="s">
+      <c r="A17" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="B17" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="C17" s="3">
-        <v>94655.86319999999</v>
+      <c r="C17" s="5">
+        <v>359</v>
       </c>
     </row>
     <row r="18" spans="1:3">
-      <c r="A18" s="2" t="s">
+      <c r="A18" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="B18" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="C18" s="3">
-        <v>3252.08</v>
+      <c r="C18" s="5">
+        <v>3325</v>
       </c>
     </row>
     <row r="19" spans="1:3">
@@ -1490,18 +1468,18 @@
         <v>38</v>
       </c>
       <c r="C19" s="5">
-        <v>95</v>
+        <v>1331.66</v>
       </c>
     </row>
     <row r="20" spans="1:3">
-      <c r="A20" s="4" t="s">
+      <c r="A20" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B20" s="4" t="s">
+      <c r="B20" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="C20" s="5">
-        <v>593.75</v>
+      <c r="C20" s="3">
+        <v>82086.21950000001</v>
       </c>
     </row>
     <row r="21" spans="1:3">
@@ -1512,7 +1490,7 @@
         <v>42</v>
       </c>
       <c r="C21" s="5">
-        <v>1993.33</v>
+        <v>82084.8395</v>
       </c>
     </row>
     <row r="22" spans="1:3">
@@ -1523,7 +1501,7 @@
         <v>44</v>
       </c>
       <c r="C22" s="5">
-        <v>570</v>
+        <v>1.38</v>
       </c>
     </row>
     <row r="23" spans="1:3">
@@ -1534,18 +1512,18 @@
         <v>46</v>
       </c>
       <c r="C23" s="3">
-        <v>62068.00999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:3">
-      <c r="A24" s="4" t="s">
+      <c r="A24" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="B24" s="4" t="s">
+      <c r="B24" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="C24" s="5">
-        <v>61616.63</v>
+      <c r="C24" s="3">
+        <v>1130</v>
       </c>
     </row>
     <row r="25" spans="1:3">
@@ -1556,29 +1534,29 @@
         <v>50</v>
       </c>
       <c r="C25" s="5">
-        <v>450</v>
+        <v>1130</v>
       </c>
     </row>
     <row r="26" spans="1:3">
-      <c r="A26" s="4" t="s">
+      <c r="A26" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="B26" s="4" t="s">
+      <c r="B26" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="C26" s="5">
-        <v>1.38</v>
+      <c r="C26" s="3">
+        <v>1639.31</v>
       </c>
     </row>
     <row r="27" spans="1:3">
-      <c r="A27" s="2" t="s">
+      <c r="A27" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="B27" s="2" t="s">
+      <c r="B27" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="C27" s="3">
-        <v>750</v>
+      <c r="C27" s="5">
+        <v>71.87</v>
       </c>
     </row>
     <row r="28" spans="1:3">
@@ -1589,18 +1567,18 @@
         <v>56</v>
       </c>
       <c r="C28" s="5">
-        <v>750</v>
+        <v>335</v>
       </c>
     </row>
     <row r="29" spans="1:3">
-      <c r="A29" s="2" t="s">
+      <c r="A29" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="B29" s="2" t="s">
+      <c r="B29" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="C29" s="3">
-        <v>4244.25</v>
+      <c r="C29" s="5">
+        <v>298.5</v>
       </c>
     </row>
     <row r="30" spans="1:3">
@@ -1611,7 +1589,7 @@
         <v>60</v>
       </c>
       <c r="C30" s="5">
-        <v>3992.5</v>
+        <v>758.9400000000001</v>
       </c>
     </row>
     <row r="31" spans="1:3">
@@ -1622,29 +1600,29 @@
         <v>62</v>
       </c>
       <c r="C31" s="5">
-        <v>251.75</v>
+        <v>150</v>
       </c>
     </row>
     <row r="32" spans="1:3">
-      <c r="A32" s="2" t="s">
+      <c r="A32" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="B32" s="2" t="s">
+      <c r="B32" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="C32" s="3">
-        <v>22636.7032</v>
+      <c r="C32" s="5">
+        <v>25</v>
       </c>
     </row>
     <row r="33" spans="1:3">
-      <c r="A33" s="4" t="s">
+      <c r="A33" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="B33" s="4" t="s">
+      <c r="B33" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="C33" s="5">
-        <v>3729.5832</v>
+      <c r="C33" s="3">
+        <v>1806.3905</v>
       </c>
     </row>
     <row r="34" spans="1:3">
@@ -1655,7 +1633,7 @@
         <v>68</v>
       </c>
       <c r="C34" s="5">
-        <v>4282.8</v>
+        <v>483.3478</v>
       </c>
     </row>
     <row r="35" spans="1:3">
@@ -1666,18 +1644,18 @@
         <v>70</v>
       </c>
       <c r="C35" s="5">
-        <v>6634.5</v>
+        <v>1323.0427</v>
       </c>
     </row>
     <row r="36" spans="1:3">
-      <c r="A36" s="4" t="s">
+      <c r="A36" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="B36" s="4" t="s">
+      <c r="B36" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="C36" s="5">
-        <v>66</v>
+      <c r="C36" s="3">
+        <v>96.70999999999999</v>
       </c>
     </row>
     <row r="37" spans="1:3">
@@ -1688,7 +1666,7 @@
         <v>74</v>
       </c>
       <c r="C37" s="5">
-        <v>557.88</v>
+        <v>95.59999999999999</v>
       </c>
     </row>
     <row r="38" spans="1:3">
@@ -1699,73 +1677,73 @@
         <v>76</v>
       </c>
       <c r="C38" s="5">
-        <v>1391.94</v>
+        <v>1.11</v>
       </c>
     </row>
     <row r="39" spans="1:3">
-      <c r="A39" s="4" t="s">
+      <c r="A39" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="B39" s="4" t="s">
+      <c r="B39" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="C39" s="5">
-        <v>924</v>
+      <c r="C39" s="3">
+        <v>0</v>
       </c>
     </row>
     <row r="40" spans="1:3">
-      <c r="A40" s="4" t="s">
+      <c r="A40" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="B40" s="4" t="s">
+      <c r="B40" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="C40" s="5">
-        <v>5050</v>
+      <c r="C40" s="3">
+        <v>818.0599999999999</v>
       </c>
     </row>
     <row r="41" spans="1:3">
-      <c r="A41" s="2" t="s">
+      <c r="A41" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="B41" s="2" t="s">
+      <c r="B41" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="C41" s="3">
-        <v>1603.2</v>
+      <c r="C41" s="5">
+        <v>818.0599999999999</v>
       </c>
     </row>
     <row r="42" spans="1:3">
-      <c r="A42" s="4" t="s">
+      <c r="A42" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="B42" s="4" t="s">
+      <c r="B42" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="C42" s="5">
-        <v>463.67</v>
+      <c r="C42" s="3">
+        <v>322663.39</v>
       </c>
     </row>
     <row r="43" spans="1:3">
-      <c r="A43" s="4" t="s">
+      <c r="A43" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="B43" s="4" t="s">
+      <c r="B43" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="C43" s="5">
-        <v>1139.53</v>
+      <c r="C43" s="3">
+        <v>5843.849999999999</v>
       </c>
     </row>
     <row r="44" spans="1:3">
-      <c r="A44" s="2" t="s">
+      <c r="A44" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="B44" s="2" t="s">
+      <c r="B44" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="C44" s="3">
-        <v>101.62</v>
+      <c r="C44" s="5">
+        <v>318.6</v>
       </c>
     </row>
     <row r="45" spans="1:3">
@@ -1776,7 +1754,7 @@
         <v>90</v>
       </c>
       <c r="C45" s="5">
-        <v>100</v>
+        <v>187.27</v>
       </c>
     </row>
     <row r="46" spans="1:3">
@@ -1787,29 +1765,29 @@
         <v>92</v>
       </c>
       <c r="C46" s="5">
-        <v>1.62</v>
+        <v>190.07</v>
       </c>
     </row>
     <row r="47" spans="1:3">
-      <c r="A47" s="2" t="s">
+      <c r="A47" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="B47" s="2" t="s">
+      <c r="B47" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="C47" s="3">
-        <v>0</v>
+      <c r="C47" s="5">
+        <v>1512.27</v>
       </c>
     </row>
     <row r="48" spans="1:3">
-      <c r="A48" s="2" t="s">
+      <c r="A48" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="B48" s="2" t="s">
+      <c r="B48" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="C48" s="3">
-        <v>1035.31</v>
+      <c r="C48" s="5">
+        <v>733.25</v>
       </c>
     </row>
     <row r="49" spans="1:3">
@@ -1820,7 +1798,7 @@
         <v>98</v>
       </c>
       <c r="C49" s="5">
-        <v>893.3299999999999</v>
+        <v>562.25</v>
       </c>
     </row>
     <row r="50" spans="1:3">
@@ -1831,29 +1809,29 @@
         <v>100</v>
       </c>
       <c r="C50" s="5">
-        <v>141.98</v>
+        <v>309.8</v>
       </c>
     </row>
     <row r="51" spans="1:3">
-      <c r="A51" s="2" t="s">
+      <c r="A51" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="B51" s="2" t="s">
+      <c r="B51" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="C51" s="3">
-        <v>404732.02</v>
+      <c r="C51" s="5">
+        <v>483.06</v>
       </c>
     </row>
     <row r="52" spans="1:3">
-      <c r="A52" s="2" t="s">
+      <c r="A52" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="B52" s="2" t="s">
+      <c r="B52" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="C52" s="3">
-        <v>14802.33</v>
+      <c r="C52" s="5">
+        <v>767.0700000000001</v>
       </c>
     </row>
     <row r="53" spans="1:3">
@@ -1864,7 +1842,7 @@
         <v>106</v>
       </c>
       <c r="C53" s="5">
-        <v>1198.67</v>
+        <v>272.74</v>
       </c>
     </row>
     <row r="54" spans="1:3">
@@ -1875,7 +1853,7 @@
         <v>108</v>
       </c>
       <c r="C54" s="5">
-        <v>1262.96</v>
+        <v>291</v>
       </c>
     </row>
     <row r="55" spans="1:3">
@@ -1886,18 +1864,18 @@
         <v>110</v>
       </c>
       <c r="C55" s="5">
-        <v>1147.55</v>
+        <v>216.47</v>
       </c>
     </row>
     <row r="56" spans="1:3">
-      <c r="A56" s="4" t="s">
+      <c r="A56" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="B56" s="4" t="s">
+      <c r="B56" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="C56" s="5">
-        <v>3541.25</v>
+      <c r="C56" s="3">
+        <v>17373.75</v>
       </c>
     </row>
     <row r="57" spans="1:3">
@@ -1908,7 +1886,7 @@
         <v>114</v>
       </c>
       <c r="C57" s="5">
-        <v>759.87</v>
+        <v>927.6</v>
       </c>
     </row>
     <row r="58" spans="1:3">
@@ -1919,7 +1897,7 @@
         <v>116</v>
       </c>
       <c r="C58" s="5">
-        <v>745.9299999999999</v>
+        <v>250</v>
       </c>
     </row>
     <row r="59" spans="1:3">
@@ -1930,7 +1908,7 @@
         <v>118</v>
       </c>
       <c r="C59" s="5">
-        <v>303.68</v>
+        <v>7155.57</v>
       </c>
     </row>
     <row r="60" spans="1:3">
@@ -1941,7 +1919,7 @@
         <v>120</v>
       </c>
       <c r="C60" s="5">
-        <v>522.76</v>
+        <v>65</v>
       </c>
     </row>
     <row r="61" spans="1:3">
@@ -1952,7 +1930,7 @@
         <v>122</v>
       </c>
       <c r="C61" s="5">
-        <v>4531.94</v>
+        <v>25</v>
       </c>
     </row>
     <row r="62" spans="1:3">
@@ -1963,7 +1941,7 @@
         <v>124</v>
       </c>
       <c r="C62" s="5">
-        <v>280.25</v>
+        <v>564.76</v>
       </c>
     </row>
     <row r="63" spans="1:3">
@@ -1974,7 +1952,7 @@
         <v>126</v>
       </c>
       <c r="C63" s="5">
-        <v>291</v>
+        <v>900.62</v>
       </c>
     </row>
     <row r="64" spans="1:3">
@@ -1985,18 +1963,18 @@
         <v>128</v>
       </c>
       <c r="C64" s="5">
-        <v>216.47</v>
+        <v>856.45</v>
       </c>
     </row>
     <row r="65" spans="1:3">
-      <c r="A65" s="2" t="s">
+      <c r="A65" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="B65" s="2" t="s">
+      <c r="B65" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="C65" s="3">
-        <v>54605.1</v>
+      <c r="C65" s="5">
+        <v>2832.19</v>
       </c>
     </row>
     <row r="66" spans="1:3">
@@ -2007,7 +1985,7 @@
         <v>132</v>
       </c>
       <c r="C66" s="5">
-        <v>147.9</v>
+        <v>1398.43</v>
       </c>
     </row>
     <row r="67" spans="1:3">
@@ -2018,18 +1996,18 @@
         <v>134</v>
       </c>
       <c r="C67" s="5">
-        <v>984.9200000000001</v>
+        <v>759</v>
       </c>
     </row>
     <row r="68" spans="1:3">
-      <c r="A68" s="4" t="s">
+      <c r="A68" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="B68" s="4" t="s">
+      <c r="B68" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="C68" s="5">
-        <v>2590.93</v>
+      <c r="C68" s="3">
+        <v>1639.13</v>
       </c>
     </row>
     <row r="69" spans="1:3">
@@ -2040,18 +2018,18 @@
         <v>138</v>
       </c>
       <c r="C69" s="5">
-        <v>1552.1</v>
+        <v>1639.13</v>
       </c>
     </row>
     <row r="70" spans="1:3">
-      <c r="A70" s="4" t="s">
+      <c r="A70" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="B70" s="4" t="s">
+      <c r="B70" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="C70" s="5">
-        <v>1113.44</v>
+      <c r="C70" s="3">
+        <v>43997.74999999999</v>
       </c>
     </row>
     <row r="71" spans="1:3">
@@ -2062,7 +2040,7 @@
         <v>142</v>
       </c>
       <c r="C71" s="5">
-        <v>2864.8</v>
+        <v>586.4300000000001</v>
       </c>
     </row>
     <row r="72" spans="1:3">
@@ -2073,7 +2051,7 @@
         <v>144</v>
       </c>
       <c r="C72" s="5">
-        <v>50</v>
+        <v>900</v>
       </c>
     </row>
     <row r="73" spans="1:3">
@@ -2084,7 +2062,7 @@
         <v>146</v>
       </c>
       <c r="C73" s="5">
-        <v>205</v>
+        <v>1284.7</v>
       </c>
     </row>
     <row r="74" spans="1:3">
@@ -2095,7 +2073,7 @@
         <v>148</v>
       </c>
       <c r="C74" s="5">
-        <v>33.98</v>
+        <v>449.9</v>
       </c>
     </row>
     <row r="75" spans="1:3">
@@ -2106,18 +2084,18 @@
         <v>150</v>
       </c>
       <c r="C75" s="5">
-        <v>759</v>
+        <v>3071</v>
       </c>
     </row>
     <row r="76" spans="1:3">
-      <c r="A76" s="2" t="s">
+      <c r="A76" s="4" t="s">
         <v>151</v>
       </c>
-      <c r="B76" s="2" t="s">
+      <c r="B76" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="C76" s="3">
-        <v>44303.03</v>
+      <c r="C76" s="5">
+        <v>2530</v>
       </c>
     </row>
     <row r="77" spans="1:3">
@@ -2125,406 +2103,406 @@
         <v>153</v>
       </c>
       <c r="B77" s="4" t="s">
-        <v>48</v>
+        <v>154</v>
       </c>
       <c r="C77" s="5">
-        <v>41721.21</v>
+        <v>522.6799999999999</v>
       </c>
     </row>
     <row r="78" spans="1:3">
       <c r="A78" s="4" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B78" s="4" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C78" s="5">
-        <v>2581.82</v>
+        <v>4200</v>
       </c>
     </row>
     <row r="79" spans="1:3">
-      <c r="A79" s="2" t="s">
-        <v>156</v>
-      </c>
-      <c r="B79" s="2" t="s">
+      <c r="A79" s="4" t="s">
         <v>157</v>
       </c>
-      <c r="C79" s="3">
-        <v>45392.85</v>
+      <c r="B79" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="C79" s="5">
+        <v>2500</v>
       </c>
     </row>
     <row r="80" spans="1:3">
       <c r="A80" s="4" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B80" s="4" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C80" s="5">
-        <v>672.86</v>
+        <v>3467.2</v>
       </c>
     </row>
     <row r="81" spans="1:3">
       <c r="A81" s="4" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B81" s="4" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C81" s="5">
-        <v>182.39</v>
+        <v>2280.59</v>
       </c>
     </row>
     <row r="82" spans="1:3">
       <c r="A82" s="4" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B82" s="4" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C82" s="5">
-        <v>900</v>
+        <v>389.34</v>
       </c>
     </row>
     <row r="83" spans="1:3">
       <c r="A83" s="4" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B83" s="4" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C83" s="5">
-        <v>1853.61</v>
+        <v>5293.690000000001</v>
       </c>
     </row>
     <row r="84" spans="1:3">
       <c r="A84" s="4" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B84" s="4" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C84" s="5">
-        <v>3154</v>
+        <v>7139.44</v>
       </c>
     </row>
     <row r="85" spans="1:3">
       <c r="A85" s="4" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B85" s="4" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C85" s="5">
-        <v>2438</v>
+        <v>2667.25</v>
       </c>
     </row>
     <row r="86" spans="1:3">
       <c r="A86" s="4" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B86" s="4" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C86" s="5">
-        <v>522.6799999999999</v>
+        <v>1636.46</v>
       </c>
     </row>
     <row r="87" spans="1:3">
       <c r="A87" s="4" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B87" s="4" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C87" s="5">
-        <v>1200</v>
+        <v>4500</v>
       </c>
     </row>
     <row r="88" spans="1:3">
       <c r="A88" s="4" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B88" s="4" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C88" s="5">
-        <v>2400</v>
+        <v>75</v>
       </c>
     </row>
     <row r="89" spans="1:3">
       <c r="A89" s="4" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B89" s="4" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C89" s="5">
-        <v>2663.4</v>
+        <v>123.32</v>
       </c>
     </row>
     <row r="90" spans="1:3">
       <c r="A90" s="4" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B90" s="4" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C90" s="5">
-        <v>2171.95</v>
+        <v>380.75</v>
       </c>
     </row>
     <row r="91" spans="1:3">
-      <c r="A91" s="4" t="s">
-        <v>180</v>
-      </c>
-      <c r="B91" s="4" t="s">
+      <c r="A91" s="2" t="s">
         <v>181</v>
       </c>
-      <c r="C91" s="5">
-        <v>378</v>
+      <c r="B91" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="C91" s="3">
+        <v>175441.3099999999</v>
       </c>
     </row>
     <row r="92" spans="1:3">
       <c r="A92" s="4" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B92" s="4" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C92" s="5">
-        <v>3239.36</v>
+        <v>60683.31</v>
       </c>
     </row>
     <row r="93" spans="1:3">
       <c r="A93" s="4" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B93" s="4" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C93" s="5">
-        <v>4369.96</v>
+        <v>48246.74</v>
       </c>
     </row>
     <row r="94" spans="1:3">
       <c r="A94" s="4" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B94" s="4" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="C94" s="5">
-        <v>6998.71</v>
+        <v>14687.87</v>
       </c>
     </row>
     <row r="95" spans="1:3">
       <c r="A95" s="4" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B95" s="4" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C95" s="5">
-        <v>2667.25</v>
+        <v>0</v>
       </c>
     </row>
     <row r="96" spans="1:3">
       <c r="A96" s="4" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B96" s="4" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="C96" s="5">
-        <v>1636.46</v>
+        <v>5033.1</v>
       </c>
     </row>
     <row r="97" spans="1:3">
       <c r="A97" s="4" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B97" s="4" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C97" s="5">
-        <v>5634.9</v>
+        <v>21732.32</v>
       </c>
     </row>
     <row r="98" spans="1:3">
       <c r="A98" s="4" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B98" s="4" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C98" s="5">
-        <v>1800</v>
+        <v>8084.92</v>
       </c>
     </row>
     <row r="99" spans="1:3">
       <c r="A99" s="4" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B99" s="4" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C99" s="5">
-        <v>129.32</v>
+        <v>351.46</v>
       </c>
     </row>
     <row r="100" spans="1:3">
       <c r="A100" s="4" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B100" s="4" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C100" s="5">
-        <v>380</v>
+        <v>666.52</v>
       </c>
     </row>
     <row r="101" spans="1:3">
-      <c r="A101" s="2" t="s">
-        <v>200</v>
-      </c>
-      <c r="B101" s="2" t="s">
+      <c r="A101" s="4" t="s">
         <v>201</v>
       </c>
-      <c r="C101" s="3">
-        <v>180985.46</v>
+      <c r="B101" s="4" t="s">
+        <v>202</v>
+      </c>
+      <c r="C101" s="5">
+        <v>399.8</v>
       </c>
     </row>
     <row r="102" spans="1:3">
       <c r="A102" s="4" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B102" s="4" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="C102" s="5">
-        <v>52637.77</v>
+        <v>430.96</v>
       </c>
     </row>
     <row r="103" spans="1:3">
       <c r="A103" s="4" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B103" s="4" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="C103" s="5">
-        <v>78823.90000000001</v>
+        <v>10921.2</v>
       </c>
     </row>
     <row r="104" spans="1:3">
       <c r="A104" s="4" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B104" s="4" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="C104" s="5">
-        <v>13558.66</v>
+        <v>4203.11</v>
       </c>
     </row>
     <row r="105" spans="1:3">
-      <c r="A105" s="4" t="s">
-        <v>208</v>
-      </c>
-      <c r="B105" s="4" t="s">
+      <c r="A105" s="2" t="s">
         <v>209</v>
       </c>
-      <c r="C105" s="5">
-        <v>0</v>
+      <c r="B105" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="C105" s="3">
+        <v>3821</v>
       </c>
     </row>
     <row r="106" spans="1:3">
       <c r="A106" s="4" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B106" s="4" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C106" s="5">
-        <v>4838.84</v>
+        <v>2621</v>
       </c>
     </row>
     <row r="107" spans="1:3">
       <c r="A107" s="4" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B107" s="4" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C107" s="5">
-        <v>20162.3</v>
+        <v>800</v>
       </c>
     </row>
     <row r="108" spans="1:3">
       <c r="A108" s="4" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B108" s="4" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C108" s="5">
-        <v>351.46</v>
+        <v>400</v>
       </c>
     </row>
     <row r="109" spans="1:3">
-      <c r="A109" s="4" t="s">
-        <v>216</v>
-      </c>
-      <c r="B109" s="4" t="s">
+      <c r="A109" s="2" t="s">
         <v>217</v>
       </c>
-      <c r="C109" s="5">
-        <v>723.52</v>
+      <c r="B109" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="C109" s="3">
+        <v>4369.84</v>
       </c>
     </row>
     <row r="110" spans="1:3">
       <c r="A110" s="4" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B110" s="4" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="C110" s="5">
-        <v>413.57</v>
+        <v>4319.84</v>
       </c>
     </row>
     <row r="111" spans="1:3">
       <c r="A111" s="4" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B111" s="4" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="C111" s="5">
-        <v>544.46</v>
+        <v>50</v>
       </c>
     </row>
     <row r="112" spans="1:3">
-      <c r="A112" s="4" t="s">
-        <v>222</v>
-      </c>
-      <c r="B112" s="4" t="s">
+      <c r="A112" s="2" t="s">
         <v>223</v>
       </c>
-      <c r="C112" s="5">
-        <v>8930.98</v>
+      <c r="B112" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="C112" s="3">
+        <v>1866.34</v>
       </c>
     </row>
     <row r="113" spans="1:3">
-      <c r="A113" s="2" t="s">
+      <c r="A113" s="4" t="s">
         <v>224</v>
       </c>
-      <c r="B113" s="2" t="s">
+      <c r="B113" s="4" t="s">
         <v>225</v>
       </c>
-      <c r="C113" s="3">
-        <v>1633.71</v>
+      <c r="C113" s="5">
+        <v>0</v>
       </c>
     </row>
     <row r="114" spans="1:3">
@@ -2535,7 +2513,7 @@
         <v>227</v>
       </c>
       <c r="C114" s="5">
-        <v>820</v>
+        <v>1269.64</v>
       </c>
     </row>
     <row r="115" spans="1:3">
@@ -2546,7 +2524,7 @@
         <v>229</v>
       </c>
       <c r="C115" s="5">
-        <v>813.7099999999999</v>
+        <v>596.7</v>
       </c>
     </row>
     <row r="116" spans="1:3">
@@ -2557,7 +2535,7 @@
         <v>231</v>
       </c>
       <c r="C116" s="3">
-        <v>8741.900000000001</v>
+        <v>29845.73</v>
       </c>
     </row>
     <row r="117" spans="1:3">
@@ -2568,164 +2546,164 @@
         <v>233</v>
       </c>
       <c r="C117" s="5">
-        <v>8741.900000000001</v>
+        <v>29010.36</v>
       </c>
     </row>
     <row r="118" spans="1:3">
-      <c r="A118" s="2" t="s">
+      <c r="A118" s="4" t="s">
         <v>234</v>
       </c>
-      <c r="B118" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="C118" s="3">
-        <v>673.46</v>
+      <c r="B118" s="4" t="s">
+        <v>235</v>
+      </c>
+      <c r="C118" s="5">
+        <v>824.45</v>
       </c>
     </row>
     <row r="119" spans="1:3">
       <c r="A119" s="4" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B119" s="4" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C119" s="5">
-        <v>673.46</v>
+        <v>10.92</v>
       </c>
     </row>
     <row r="120" spans="1:3">
       <c r="A120" s="2" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B120" s="2" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="C120" s="3">
-        <v>34628.66</v>
+        <v>1775.5</v>
       </c>
     </row>
     <row r="121" spans="1:3">
       <c r="A121" s="4" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B121" s="4" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C121" s="5">
-        <v>575.7</v>
+        <v>538.65</v>
       </c>
     </row>
     <row r="122" spans="1:3">
       <c r="A122" s="4" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B122" s="4" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="C122" s="5">
-        <v>2035.67</v>
+        <v>454.67</v>
       </c>
     </row>
     <row r="123" spans="1:3">
       <c r="A123" s="4" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="B123" s="4" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="C123" s="5">
-        <v>2603.42</v>
+        <v>782.1799999999999</v>
       </c>
     </row>
     <row r="124" spans="1:3">
-      <c r="A124" s="4" t="s">
-        <v>245</v>
-      </c>
-      <c r="B124" s="4" t="s">
+      <c r="A124" s="2" t="s">
         <v>246</v>
       </c>
-      <c r="C124" s="5">
-        <v>29402.95</v>
+      <c r="B124" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="C124" s="3">
+        <v>1474.64</v>
       </c>
     </row>
     <row r="125" spans="1:3">
       <c r="A125" s="4" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B125" s="4" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C125" s="5">
-        <v>10.92</v>
+        <v>1474.64</v>
       </c>
     </row>
     <row r="126" spans="1:3">
       <c r="A126" s="2" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="B126" s="2" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C126" s="3">
-        <v>782.1799999999999</v>
+        <v>19787.77</v>
       </c>
     </row>
     <row r="127" spans="1:3">
       <c r="A127" s="4" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="B127" s="4" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C127" s="5">
-        <v>782.1799999999999</v>
+        <v>19787.77</v>
       </c>
     </row>
     <row r="128" spans="1:3">
       <c r="A128" s="2" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="B128" s="2" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C128" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="129" spans="1:3">
-      <c r="A129" s="2" t="s">
-        <v>255</v>
-      </c>
-      <c r="B129" s="2" t="s">
+        <v>269.04</v>
+      </c>
+    </row>
+    <row r="129" spans="1:5">
+      <c r="A129" s="4" t="s">
         <v>256</v>
       </c>
-      <c r="C129" s="3">
-        <v>21763.02</v>
-      </c>
-    </row>
-    <row r="130" spans="1:3">
+      <c r="B129" s="4" t="s">
+        <v>257</v>
+      </c>
+      <c r="C129" s="5">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="130" spans="1:5">
       <c r="A130" s="4" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B130" s="4" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C130" s="5">
-        <v>21763.02</v>
-      </c>
-    </row>
-    <row r="131" spans="1:3">
+        <v>149.04</v>
+      </c>
+    </row>
+    <row r="131" spans="1:5">
       <c r="A131" s="2" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B131" s="2" t="s">
-        <v>260</v>
+        <v>52</v>
       </c>
       <c r="C131" s="3">
-        <v>1934.81</v>
-      </c>
-    </row>
-    <row r="132" spans="1:3">
+        <v>2243.34</v>
+      </c>
+    </row>
+    <row r="132" spans="1:5">
       <c r="A132" s="4" t="s">
         <v>261</v>
       </c>
@@ -2733,194 +2711,135 @@
         <v>262</v>
       </c>
       <c r="C132" s="5">
-        <v>1934.81</v>
-      </c>
-    </row>
-    <row r="133" spans="1:3">
-      <c r="A133" s="2" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="133" spans="1:5">
+      <c r="A133" s="4" t="s">
         <v>263</v>
       </c>
-      <c r="B133" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="C133" s="3">
-        <v>27098.68</v>
-      </c>
-    </row>
-    <row r="134" spans="1:3">
+      <c r="B133" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="C133" s="5">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="134" spans="1:5">
       <c r="A134" s="4" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B134" s="4" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="C134" s="5">
-        <v>5694.14</v>
-      </c>
-    </row>
-    <row r="135" spans="1:3">
-      <c r="A135" s="4" t="s">
-        <v>266</v>
-      </c>
-      <c r="B135" s="4" t="s">
+        <v>743.34</v>
+      </c>
+    </row>
+    <row r="135" spans="1:5">
+      <c r="A135" s="2" t="s">
         <v>267</v>
       </c>
-      <c r="C135" s="5">
-        <v>436.7</v>
-      </c>
-    </row>
-    <row r="136" spans="1:3">
+      <c r="B135" s="2" t="s">
+        <v>268</v>
+      </c>
+      <c r="C135" s="3">
+        <v>14553.53</v>
+      </c>
+    </row>
+    <row r="136" spans="1:5">
       <c r="A136" s="4" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="B136" s="4" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="C136" s="5">
-        <v>1670</v>
-      </c>
-    </row>
-    <row r="137" spans="1:3">
+        <v>1709.42</v>
+      </c>
+    </row>
+    <row r="137" spans="1:5">
       <c r="A137" s="4" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="B137" s="4" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C137" s="5">
-        <v>3000</v>
-      </c>
-    </row>
-    <row r="138" spans="1:3">
+        <v>3852.01</v>
+      </c>
+    </row>
+    <row r="138" spans="1:5">
       <c r="A138" s="4" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="B138" s="4" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C138" s="5">
-        <v>3250</v>
-      </c>
-    </row>
-    <row r="139" spans="1:3">
+        <v>5896.28</v>
+      </c>
+    </row>
+    <row r="139" spans="1:5">
       <c r="A139" s="4" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="B139" s="4" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C139" s="5">
+        <v>3095.82</v>
+      </c>
+    </row>
+    <row r="141" spans="1:5">
+      <c r="A141" s="6" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="140" spans="1:3">
-      <c r="A140" s="4" t="s">
-        <v>276</v>
-      </c>
-      <c r="B140" s="4" t="s">
+      <c r="B141" s="6" t="s">
         <v>277</v>
       </c>
-      <c r="C140" s="5">
-        <v>2100</v>
-      </c>
-    </row>
-    <row r="141" spans="1:3">
-      <c r="A141" s="4" t="s">
+      <c r="C141" s="6" t="s">
         <v>278</v>
       </c>
-      <c r="B141" s="4" t="s">
+      <c r="D141" s="6" t="s">
         <v>279</v>
       </c>
-      <c r="C141" s="5">
-        <v>8892</v>
-      </c>
-    </row>
-    <row r="142" spans="1:3">
-      <c r="A142" s="4" t="s">
+      <c r="E141" s="6" t="s">
         <v>280</v>
       </c>
-      <c r="B142" s="4" t="s">
-        <v>281</v>
-      </c>
-      <c r="C142" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="143" spans="1:3">
-      <c r="A143" s="4" t="s">
-        <v>282</v>
-      </c>
-      <c r="B143" s="4" t="s">
-        <v>283</v>
-      </c>
-      <c r="C143" s="5">
-        <v>1312.5</v>
-      </c>
-    </row>
-    <row r="144" spans="1:3">
-      <c r="A144" s="4" t="s">
-        <v>284</v>
-      </c>
-      <c r="B144" s="4" t="s">
-        <v>285</v>
-      </c>
-      <c r="C144" s="5">
-        <v>743.34</v>
-      </c>
-    </row>
-    <row r="145" spans="1:3">
-      <c r="A145" s="2" t="s">
-        <v>286</v>
-      </c>
-      <c r="B145" s="2" t="s">
-        <v>287</v>
-      </c>
-      <c r="C145" s="3">
-        <v>11689.86</v>
-      </c>
-    </row>
-    <row r="146" spans="1:3">
-      <c r="A146" s="4" t="s">
-        <v>288</v>
-      </c>
-      <c r="B146" s="4" t="s">
-        <v>289</v>
-      </c>
-      <c r="C146" s="5">
-        <v>1709.42</v>
-      </c>
-    </row>
-    <row r="147" spans="1:3">
-      <c r="A147" s="4" t="s">
-        <v>290</v>
-      </c>
-      <c r="B147" s="4" t="s">
-        <v>291</v>
-      </c>
-      <c r="C147" s="5">
-        <v>920.66</v>
-      </c>
-    </row>
-    <row r="148" spans="1:3">
-      <c r="A148" s="4" t="s">
-        <v>292</v>
-      </c>
-      <c r="B148" s="4" t="s">
-        <v>293</v>
-      </c>
-      <c r="C148" s="5">
-        <v>5465.2</v>
-      </c>
-    </row>
-    <row r="149" spans="1:3">
-      <c r="A149" s="4" t="s">
-        <v>294</v>
-      </c>
-      <c r="B149" s="4" t="s">
-        <v>295</v>
-      </c>
-      <c r="C149" s="5">
-        <v>3594.58</v>
+    </row>
+    <row r="142" spans="1:5">
+      <c r="A142" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B142" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="C142" s="7">
+        <v>379129.2</v>
+      </c>
+      <c r="D142" s="7">
+        <v>438415</v>
+      </c>
+      <c r="E142" s="8">
+        <v>-59285.8</v>
+      </c>
+    </row>
+    <row r="143" spans="1:5">
+      <c r="A143" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="B143" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="C143" s="7">
+        <v>322663.39</v>
+      </c>
+      <c r="D143" s="7">
+        <v>446163.39</v>
+      </c>
+      <c r="E143" s="8">
+        <v>-123500</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
changing column of paid accounts to valor_class
</commit_message>
<xml_diff>
--- a/fluxo_de_caixa.xlsx
+++ b/fluxo_de_caixa.xlsx
@@ -1875,7 +1875,7 @@
         <v>112</v>
       </c>
       <c r="C56" s="3">
-        <v>17373.75</v>
+        <v>17218.43</v>
       </c>
     </row>
     <row r="57" spans="1:3">
@@ -1908,7 +1908,7 @@
         <v>118</v>
       </c>
       <c r="C59" s="5">
-        <v>7155.57</v>
+        <v>7000.25</v>
       </c>
     </row>
     <row r="60" spans="1:3">
@@ -2029,7 +2029,7 @@
         <v>140</v>
       </c>
       <c r="C70" s="3">
-        <v>43997.74999999999</v>
+        <v>43992.16</v>
       </c>
     </row>
     <row r="71" spans="1:3">
@@ -2150,7 +2150,7 @@
         <v>162</v>
       </c>
       <c r="C81" s="5">
-        <v>2280.59</v>
+        <v>2275</v>
       </c>
     </row>
     <row r="82" spans="1:3">
@@ -2293,7 +2293,7 @@
         <v>188</v>
       </c>
       <c r="C94" s="5">
-        <v>14687.87</v>
+        <v>7343.94</v>
       </c>
     </row>
     <row r="95" spans="1:3">
@@ -2304,7 +2304,7 @@
         <v>190</v>
       </c>
       <c r="C95" s="5">
-        <v>0</v>
+        <v>7343.93</v>
       </c>
     </row>
     <row r="96" spans="1:3">
@@ -2491,7 +2491,7 @@
         <v>66</v>
       </c>
       <c r="C112" s="3">
-        <v>1866.34</v>
+        <v>1871.93</v>
       </c>
     </row>
     <row r="113" spans="1:3">
@@ -2502,7 +2502,7 @@
         <v>225</v>
       </c>
       <c r="C113" s="5">
-        <v>0</v>
+        <v>5.59</v>
       </c>
     </row>
     <row r="114" spans="1:3">
@@ -2700,7 +2700,7 @@
         <v>52</v>
       </c>
       <c r="C131" s="3">
-        <v>2243.34</v>
+        <v>2250.46</v>
       </c>
     </row>
     <row r="132" spans="1:5">
@@ -2711,7 +2711,7 @@
         <v>262</v>
       </c>
       <c r="C132" s="5">
-        <v>0</v>
+        <v>7.12</v>
       </c>
     </row>
     <row r="133" spans="1:5">
@@ -2744,7 +2744,7 @@
         <v>268</v>
       </c>
       <c r="C135" s="3">
-        <v>14553.53</v>
+        <v>14701.73</v>
       </c>
     </row>
     <row r="136" spans="1:5">
@@ -2788,7 +2788,7 @@
         <v>276</v>
       </c>
       <c r="C139" s="5">
-        <v>3095.82</v>
+        <v>3244.02</v>
       </c>
     </row>
     <row r="141" spans="1:5">

</xml_diff>